<commit_message>
feat: Add Kaizen image, Pareto Ishikawa template, and LEAN guide PDF.
</commit_message>
<xml_diff>
--- a/OI/a0_pareto_ishikawa/Template_Pareto_Chaudronnier.xlsx
+++ b/OI/a0_pareto_ishikawa/Template_Pareto_Chaudronnier.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/A0 Pareto - Ishikawa/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/a0_pareto_ishikawa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="11_E62DBA95E96421727B015E18D07CDFF7B80D98E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{605B835E-AB6D-4020-A746-167E53F7C4B8}"/>
+  <xr:revisionPtr revIDLastSave="51" documentId="11_E62DBA95E96421727B015E18D07CDFF7B80D98E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CA44984-C7E9-443D-B1D5-F6C69FD7DBB3}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Modele Vierge" sheetId="1" r:id="rId1"/>
@@ -392,11 +392,6 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -414,6 +409,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1267,16 +1267,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>997164</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>129945</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>64405</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>65787</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>643801</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>64997</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>703023</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>188378</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1302,10 +1302,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1597,51 +1593,51 @@
     <tabColor rgb="FFE67E22"/>
   </sheetPr>
   <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
@@ -1655,67 +1651,67 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>11</v>
       </c>
@@ -1737,122 +1733,122 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC1EFDFC-80EF-46B3-B4F8-F8369B7E5EB6}">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.265625" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="17" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A2" s="15" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="16">
+      <c r="B2" s="13">
         <v>42</v>
       </c>
-      <c r="C2" s="18">
+      <c r="C2" s="15">
         <f>B2/$B$8</f>
         <v>0.56756756756756754</v>
       </c>
-      <c r="D2" s="21">
+      <c r="D2" s="18">
         <f>C2</f>
         <v>0.56756756756756754</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A3" s="17" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="B3" s="16">
+      <c r="B3" s="13">
         <v>13</v>
       </c>
-      <c r="C3" s="18">
+      <c r="C3" s="15">
         <f t="shared" ref="C3:C7" si="0">B3/$B$8</f>
         <v>0.17567567567567569</v>
       </c>
-      <c r="D3" s="21">
+      <c r="D3" s="18">
         <f>D2+C3</f>
         <v>0.7432432432432432</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="23.65" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="15" t="s">
+    <row r="4" spans="1:4" ht="23.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="B4" s="16">
+      <c r="B4" s="13">
         <v>8</v>
       </c>
-      <c r="C4" s="18">
+      <c r="C4" s="15">
         <f t="shared" si="0"/>
         <v>0.10810810810810811</v>
       </c>
-      <c r="D4" s="21">
+      <c r="D4" s="18">
         <f t="shared" ref="D4:D7" si="1">D3+C4</f>
         <v>0.85135135135135132</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="27" x14ac:dyDescent="0.45">
-      <c r="A5" s="17" t="s">
+    <row r="5" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="B5" s="16">
+      <c r="B5" s="13">
         <v>5</v>
       </c>
-      <c r="C5" s="18">
+      <c r="C5" s="15">
         <f t="shared" si="0"/>
         <v>6.7567567567567571E-2</v>
       </c>
-      <c r="D5" s="21">
+      <c r="D5" s="18">
         <f t="shared" si="1"/>
         <v>0.91891891891891886</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A6" s="15" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B6" s="16">
+      <c r="B6" s="13">
         <v>3</v>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="15">
         <f t="shared" si="0"/>
         <v>4.0540540540540543E-2</v>
       </c>
-      <c r="D6" s="21">
+      <c r="D6" s="18">
         <f t="shared" si="1"/>
         <v>0.95945945945945943</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A7" s="17" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="13">
         <v>3</v>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="15">
         <f t="shared" si="0"/>
         <v>4.0540540540540543E-2</v>
       </c>
-      <c r="D7" s="21">
+      <c r="D7" s="18">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B8">
         <f>SUM(B2:B7)</f>
         <v>74</v>
@@ -1871,31 +1867,31 @@
     <tabColor rgb="FFD35400"/>
   </sheetPr>
   <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>7</v>
       </c>
@@ -1906,7 +1902,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
@@ -1917,7 +1913,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>18</v>
       </c>
@@ -1928,7 +1924,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>20</v>
       </c>
@@ -1939,7 +1935,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -1950,7 +1946,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>24</v>
       </c>
@@ -1961,7 +1957,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>26</v>
       </c>
@@ -1972,7 +1968,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>28</v>
       </c>
@@ -1983,7 +1979,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>30</v>
       </c>
@@ -1994,7 +1990,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>11</v>
       </c>
@@ -2003,7 +1999,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
@@ -2022,29 +2018,29 @@
     <tabColor rgb="FF8E44AD"/>
   </sheetPr>
   <dimension ref="A1:E22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="11" max="11" width="28.73046875" customWidth="1"/>
-    <col min="12" max="12" width="20.73046875" customWidth="1"/>
+    <col min="11" max="11" width="28.7109375" customWidth="1"/>
+    <col min="12" max="12" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-    </row>
-    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+    </row>
+    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -2052,7 +2048,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>35</v>
       </c>
@@ -2060,7 +2056,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>36</v>
       </c>
@@ -2068,7 +2064,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>37</v>
       </c>
@@ -2076,7 +2072,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>38</v>
       </c>
@@ -2084,7 +2080,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>39</v>
       </c>
@@ -2092,7 +2088,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>40</v>
       </c>
@@ -2100,7 +2096,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>41</v>
       </c>
@@ -2108,12 +2104,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>7</v>
       </c>
@@ -2121,7 +2117,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>43</v>
       </c>
@@ -2129,7 +2125,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>44</v>
       </c>
@@ -2137,7 +2133,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>45</v>
       </c>
@@ -2145,7 +2141,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>46</v>
       </c>
@@ -2153,7 +2149,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
@@ -2161,7 +2157,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>47</v>
       </c>
@@ -2169,7 +2165,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>48</v>
       </c>

</xml_diff>